<commit_message>
feat: assign-all endpoint, harita UI güncellemeleri, geocode karşılaştırma araçları
</commit_message>
<xml_diff>
--- a/Docs/geocode_results.xlsx
+++ b/Docs/geocode_results.xlsx
@@ -26,12 +26,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB347"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF9999"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CC99FF"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -46,8 +61,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -625,28 +643,28 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>E8KM</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Çeşmebaşı Mahallesi, Yayla Sokak, No: 1, Bursa</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Arapzade Mah., Yayla Sok., No:1, Orhangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="1" t="n">
         <v>40.499108</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8" s="1" t="n">
         <v>29.300296</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -709,28 +727,28 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>T11SB</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Ertuğrulgazi Mahallesi, Selçukbey Caddesi, No: 96, Bursa</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Selçukbey Cad., No:96, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="1" t="n">
         <v>40.180047</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11" s="1" t="n">
         <v>29.117758</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -765,28 +783,28 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Q13JB</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Dr. Ziya Kaya Mahallesi, Atlas Sokak, No: 9, Bursa</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Yenidoğan Mah., Atlas Sok., No:9, Gürsu, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="1" t="n">
         <v>40.206108</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13" s="1" t="n">
         <v>29.18205</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1297,28 +1315,28 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>P32TM</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="1" t="inlineStr">
         <is>
           <t>Yavuzselim Mahallesi, Ankara Caddesi, No: 273, Bursa</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="1" t="inlineStr">
         <is>
           <t>Ankarayolu Cad., No:273, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D32" t="n">
+      <c r="D32" s="1" t="n">
         <v>40.191932</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E32" s="1" t="n">
         <v>29.116222</v>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1633,20 +1651,20 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>A44PM</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Balkan Mahallesi, Palandöken Sokak, No: 1E, Bursa</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr"/>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -1793,56 +1811,56 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="1" t="inlineStr">
         <is>
           <t>R50MB</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="1" t="inlineStr">
         <is>
           <t>Yeni Mudanya Yolu, Bursa</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="1" t="inlineStr">
         <is>
           <t>Aydınpınar Mah., Yeni Mudanya Yolu Cad., Mudanya, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D50" s="1" t="n">
         <v>40.332206</v>
       </c>
-      <c r="E50" t="n">
+      <c r="E50" s="1" t="n">
         <v>28.921575</v>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="1" t="inlineStr">
         <is>
           <t>T51QM</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="1" t="inlineStr">
         <is>
           <t>Çiftehavuzlar Mahallesi, Özcan Caddesi, No: 31, Bursa</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="1" t="inlineStr">
         <is>
           <t>Özcan Cad., No:31, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D51" s="1" t="n">
         <v>40.210178</v>
       </c>
-      <c r="E51" t="n">
+      <c r="E51" s="1" t="n">
         <v>29.054409</v>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1905,28 +1923,28 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="1" t="inlineStr">
         <is>
           <t>E54OM</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="1" t="inlineStr">
         <is>
           <t>Yediselviler Mahallesi, 4. Gelincik Sokak, No: 42, Bursa</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="1" t="inlineStr">
         <is>
           <t>4. Gelincik Sok., No:42, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="D54" s="1" t="n">
         <v>40.181025</v>
       </c>
-      <c r="E54" t="n">
+      <c r="E54" s="1" t="n">
         <v>29.094465</v>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -1961,20 +1979,20 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>E56PM</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Küplüpınar Mahallesi, Özdağ Sokak, Bursa</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -2121,20 +2139,20 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>I62UB</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Mürsel Mahallesi, 21. Yüzyıl Caddesi, No: 31A, Bursa</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr"/>
-      <c r="D62" t="inlineStr"/>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -2393,28 +2411,28 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="1" t="inlineStr">
         <is>
           <t>B72NM</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="1" t="inlineStr">
         <is>
           <t>Kurtuluş Mahallesi, Tunalı Sokak, No: 7, Bursa</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="1" t="inlineStr">
         <is>
           <t>Küçükbalıklı Mah., Tunalı Sok., No:7, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D72" s="1" t="n">
         <v>40.214524</v>
       </c>
-      <c r="E72" t="n">
+      <c r="E72" s="1" t="n">
         <v>29.072285</v>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F72" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2673,28 +2691,28 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="1" t="inlineStr">
         <is>
           <t>H82JM</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
+      <c r="B82" s="1" t="inlineStr">
         <is>
           <t>Doğanbey Mahallesi, Kiremitçi Caddesi, No: 6, Bursa</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
+      <c r="C82" s="1" t="inlineStr">
         <is>
           <t>Kiremitçi Cad., No:6, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D82" t="n">
+      <c r="D82" s="1" t="n">
         <v>40.188907</v>
       </c>
-      <c r="E82" t="n">
+      <c r="E82" s="1" t="n">
         <v>29.064901</v>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="F82" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -2813,20 +2831,20 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>Q87JM</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>Akçağlayan Mahallesi, 1. Zeytin Sokak, No: 33, Bursa</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
-      <c r="D87" t="inlineStr"/>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -3085,28 +3103,28 @@
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="1" t="inlineStr">
         <is>
           <t>V97EM</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B97" s="1" t="inlineStr">
         <is>
           <t>Güneştepe Mahallesi, Birol Sokak, No: 23, Bursa</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C97" s="1" t="inlineStr">
         <is>
           <t>Değirmenlikızık Mah., 2. Birol Sok., No:23, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D97" t="n">
+      <c r="D97" s="1" t="n">
         <v>40.175272</v>
       </c>
-      <c r="E97" t="n">
+      <c r="E97" s="1" t="n">
         <v>29.1097</v>
       </c>
-      <c r="F97" t="inlineStr">
+      <c r="F97" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -3309,28 +3327,28 @@
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr">
+      <c r="A105" s="1" t="inlineStr">
         <is>
           <t>L105NM</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="1" t="inlineStr">
         <is>
           <t>75. Yıl Mahallesi, Balaban Caddesi, No: 20, Bursa</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="1" t="inlineStr">
         <is>
           <t>Balaban Cad., No:20, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D105" t="n">
+      <c r="D105" s="1" t="n">
         <v>40.181838</v>
       </c>
-      <c r="E105" t="n">
+      <c r="E105" s="1" t="n">
         <v>29.14663</v>
       </c>
-      <c r="F105" t="inlineStr">
+      <c r="F105" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -3477,20 +3495,20 @@
       </c>
     </row>
     <row r="111">
-      <c r="A111" t="inlineStr">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>M111VM</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>Piremir Mahallesi, Pakyol Sokak, No: 17A, Bursa</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
-      <c r="D111" t="inlineStr"/>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr"/>
+      <c r="D111" s="2" t="inlineStr"/>
+      <c r="E111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -3917,28 +3935,28 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
+      <c r="A127" s="1" t="inlineStr">
         <is>
           <t>S127FM</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="1" t="inlineStr">
         <is>
           <t>Yavuzselim Mahallesi, Barış Caddesi, No: 42, Bursa</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
+      <c r="C127" s="1" t="inlineStr">
         <is>
           <t>Barış Cad., No:42, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D127" t="n">
+      <c r="D127" s="1" t="n">
         <v>40.194481</v>
       </c>
-      <c r="E127" t="n">
+      <c r="E127" s="1" t="n">
         <v>29.111128</v>
       </c>
-      <c r="F127" t="inlineStr">
+      <c r="F127" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -4001,28 +4019,28 @@
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
+      <c r="A130" s="1" t="inlineStr">
         <is>
           <t>J130VM</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B130" s="1" t="inlineStr">
         <is>
           <t>Hocataşkın Mahallesi, Şible Caddesi, No: 35, Bursa</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C130" s="1" t="inlineStr">
         <is>
           <t>Yeşil Mah., Şible Cad., No:35, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D130" t="n">
+      <c r="D130" s="1" t="n">
         <v>40.181108</v>
       </c>
-      <c r="E130" t="n">
+      <c r="E130" s="1" t="n">
         <v>29.076382</v>
       </c>
-      <c r="F130" t="inlineStr">
+      <c r="F130" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -4673,28 +4691,28 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="inlineStr">
+      <c r="A154" s="1" t="inlineStr">
         <is>
           <t>Y154IM</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="1" t="inlineStr">
         <is>
           <t>75. Yıl Mahallesi, Esenevler Caddesi, No: 10, Bursa</t>
         </is>
       </c>
-      <c r="C154" t="inlineStr">
+      <c r="C154" s="1" t="inlineStr">
         <is>
           <t>Esenevler Cad., No:10, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D154" t="n">
+      <c r="D154" s="1" t="n">
         <v>40.187447</v>
       </c>
-      <c r="E154" t="n">
+      <c r="E154" s="1" t="n">
         <v>29.150475</v>
       </c>
-      <c r="F154" t="inlineStr">
+      <c r="F154" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -4813,20 +4831,20 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
+      <c r="A159" s="2" t="inlineStr">
         <is>
           <t>D159ZM</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B159" s="2" t="inlineStr">
         <is>
           <t>Doğanbey Mahallesi, Kiremitçi Caddesi, No: 16, Bursa</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr"/>
-      <c r="D159" t="inlineStr"/>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr">
+      <c r="C159" s="2" t="inlineStr"/>
+      <c r="D159" s="2" t="inlineStr"/>
+      <c r="E159" s="2" t="inlineStr"/>
+      <c r="F159" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -4945,20 +4963,20 @@
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="inlineStr">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>M164CM</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
         <is>
           <t>Yeşilova Mahallesi, Kemerçeşme Caddesi, No: 248, Bursa</t>
         </is>
       </c>
-      <c r="C164" t="inlineStr"/>
-      <c r="D164" t="inlineStr"/>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr">
+      <c r="C164" s="2" t="inlineStr"/>
+      <c r="D164" s="2" t="inlineStr"/>
+      <c r="E164" s="2" t="inlineStr"/>
+      <c r="F164" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -5049,20 +5067,20 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="inlineStr">
+      <c r="A168" s="2" t="inlineStr">
         <is>
           <t>L168MB</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B168" s="2" t="inlineStr">
         <is>
           <t>Balkan Mahallesi, Hardal Sokak, No: 1D, Bursa</t>
         </is>
       </c>
-      <c r="C168" t="inlineStr"/>
-      <c r="D168" t="inlineStr"/>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr">
+      <c r="C168" s="2" t="inlineStr"/>
+      <c r="D168" s="2" t="inlineStr"/>
+      <c r="E168" s="2" t="inlineStr"/>
+      <c r="F168" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -5377,20 +5395,20 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="inlineStr">
+      <c r="A180" s="2" t="inlineStr">
         <is>
           <t>T180VB</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr">
+      <c r="B180" s="2" t="inlineStr">
         <is>
           <t>Millet Mahallesi, Milli Sokak, No: 87, Bursa</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr"/>
-      <c r="D180" t="inlineStr"/>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr">
+      <c r="C180" s="2" t="inlineStr"/>
+      <c r="D180" s="2" t="inlineStr"/>
+      <c r="E180" s="2" t="inlineStr"/>
+      <c r="F180" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -5453,20 +5471,20 @@
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="inlineStr">
+      <c r="A183" s="2" t="inlineStr">
         <is>
           <t>P183CM</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B183" s="2" t="inlineStr">
         <is>
           <t>Fatih Mahallesi, 2. Saytuk Sokak, No: 88, Bursa</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr"/>
-      <c r="D183" t="inlineStr"/>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr">
+      <c r="C183" s="2" t="inlineStr"/>
+      <c r="D183" s="2" t="inlineStr"/>
+      <c r="E183" s="2" t="inlineStr"/>
+      <c r="F183" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -5585,28 +5603,28 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" t="inlineStr">
+      <c r="A188" s="1" t="inlineStr">
         <is>
           <t>F188JM</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
+      <c r="B188" s="1" t="inlineStr">
         <is>
           <t>Çiftehavuzlar Mahallesi, 2. Kanal Caddesi, No: 298, Bursa</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr">
+      <c r="C188" s="1" t="inlineStr">
         <is>
           <t>Soğanlı Mah., 2. Kanal Cad., No:298, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D188" t="n">
+      <c r="D188" s="1" t="n">
         <v>40.214545</v>
       </c>
-      <c r="E188" t="n">
+      <c r="E188" s="1" t="n">
         <v>29.049468</v>
       </c>
-      <c r="F188" t="inlineStr">
+      <c r="F188" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -5921,20 +5939,20 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr">
+      <c r="A200" s="2" t="inlineStr">
         <is>
           <t>Z200QM</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
+      <c r="B200" s="2" t="inlineStr">
         <is>
           <t>Değirmenlikızık Mahallesi, 4. Şahin Sokak, No: 8, Bursa</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr"/>
-      <c r="D200" t="inlineStr"/>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr">
+      <c r="C200" s="2" t="inlineStr"/>
+      <c r="D200" s="2" t="inlineStr"/>
+      <c r="E200" s="2" t="inlineStr"/>
+      <c r="F200" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -5997,28 +6015,28 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr">
+      <c r="A203" s="1" t="inlineStr">
         <is>
           <t>L203YM</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
+      <c r="B203" s="1" t="inlineStr">
         <is>
           <t>İntizam Mahallesi, Değirmen Caddesi, No: 44, Bursa</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C203" s="1" t="inlineStr">
         <is>
           <t>Değirmen Cad., No:44-48, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D203" t="n">
+      <c r="D203" s="1" t="n">
         <v>40.191642</v>
       </c>
-      <c r="E203" t="n">
+      <c r="E203" s="1" t="n">
         <v>29.054409</v>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="F203" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -6193,28 +6211,28 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr">
+      <c r="A210" s="1" t="inlineStr">
         <is>
           <t>V210PM</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
+      <c r="B210" s="1" t="inlineStr">
         <is>
           <t>Yıldırım Mahallesi, Barutluk Caddesi, No: 71, Bursa</t>
         </is>
       </c>
-      <c r="C210" t="inlineStr">
+      <c r="C210" s="1" t="inlineStr">
         <is>
           <t>Barutluk Cad., No:71, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D210" t="n">
+      <c r="D210" s="1" t="n">
         <v>40.186152</v>
       </c>
-      <c r="E210" t="n">
+      <c r="E210" s="1" t="n">
         <v>29.083739</v>
       </c>
-      <c r="F210" t="inlineStr">
+      <c r="F210" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -6249,28 +6267,28 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr">
+      <c r="A212" s="1" t="inlineStr">
         <is>
           <t>M212EM</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
+      <c r="B212" s="1" t="inlineStr">
         <is>
           <t>Çiftehavuzlar Mahallesi, Özcan Caddesi, No: 27, Bursa</t>
         </is>
       </c>
-      <c r="C212" t="inlineStr">
+      <c r="C212" s="1" t="inlineStr">
         <is>
           <t>Özcan Cad., No:27, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D212" t="n">
+      <c r="D212" s="1" t="n">
         <v>40.210068</v>
       </c>
-      <c r="E212" t="n">
+      <c r="E212" s="1" t="n">
         <v>29.054427</v>
       </c>
-      <c r="F212" t="inlineStr">
+      <c r="F212" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -6557,28 +6575,28 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" t="inlineStr">
+      <c r="A223" s="1" t="inlineStr">
         <is>
           <t>B223FB</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr">
+      <c r="B223" s="1" t="inlineStr">
         <is>
           <t>Görükle Mahallesi, Ferah Sokak, No: 16, Bursa</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr">
+      <c r="C223" s="1" t="inlineStr">
         <is>
           <t>Alemdar Mah., 1. Ferah Sok., No:16, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D223" t="n">
+      <c r="D223" s="1" t="n">
         <v>40.206239</v>
       </c>
-      <c r="E223" t="n">
+      <c r="E223" s="1" t="n">
         <v>29.033245</v>
       </c>
-      <c r="F223" t="inlineStr">
+      <c r="F223" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -6697,28 +6715,28 @@
       </c>
     </row>
     <row r="228">
-      <c r="A228" t="inlineStr">
+      <c r="A228" s="1" t="inlineStr">
         <is>
           <t>C228SM</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
+      <c r="B228" s="1" t="inlineStr">
         <is>
           <t>Akçağlayan Mahallesi, Işık Caddesi, No: 30A, Bursa</t>
         </is>
       </c>
-      <c r="C228" t="inlineStr">
+      <c r="C228" s="1" t="inlineStr">
         <is>
           <t>Piremir Mah., Işık Cad., No:30А, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D228" t="n">
+      <c r="D228" s="1" t="n">
         <v>40.174383</v>
       </c>
-      <c r="E228" t="n">
+      <c r="E228" s="1" t="n">
         <v>29.084808</v>
       </c>
-      <c r="F228" t="inlineStr">
+      <c r="F228" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -6921,28 +6939,28 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" t="inlineStr">
+      <c r="A236" s="1" t="inlineStr">
         <is>
           <t>A236SM</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
+      <c r="B236" s="1" t="inlineStr">
         <is>
           <t>Namazgah Mahallesi, Işıklar Caddesi, No: 24, Bursa</t>
         </is>
       </c>
-      <c r="C236" t="inlineStr">
+      <c r="C236" s="1" t="inlineStr">
         <is>
           <t>Işıklar Cad., No:24, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D236" t="n">
+      <c r="D236" s="1" t="n">
         <v>40.177263</v>
       </c>
-      <c r="E236" t="n">
+      <c r="E236" s="1" t="n">
         <v>29.075061</v>
       </c>
-      <c r="F236" t="inlineStr">
+      <c r="F236" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -7033,20 +7051,20 @@
       </c>
     </row>
     <row r="240">
-      <c r="A240" t="inlineStr">
+      <c r="A240" s="2" t="inlineStr">
         <is>
           <t>T240BM</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
+      <c r="B240" s="2" t="inlineStr">
         <is>
           <t>Güzelyalı Siteler Mahallesi, Bursa Asfaltı Caddesi, No: 154, Bursa</t>
         </is>
       </c>
-      <c r="C240" t="inlineStr"/>
-      <c r="D240" t="inlineStr"/>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr">
+      <c r="C240" s="2" t="inlineStr"/>
+      <c r="D240" s="2" t="inlineStr"/>
+      <c r="E240" s="2" t="inlineStr"/>
+      <c r="F240" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -7137,28 +7155,28 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" t="inlineStr">
+      <c r="A244" s="1" t="inlineStr">
         <is>
           <t>Z244UM</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
+      <c r="B244" s="1" t="inlineStr">
         <is>
           <t>Küplüpınar Mahallesi, Doktor Sadık Ahmet Caddesi, No: 278, Bursa</t>
         </is>
       </c>
-      <c r="C244" t="inlineStr">
+      <c r="C244" s="1" t="inlineStr">
         <is>
           <t>Dr. Sadık Ahmet Cad., No:278, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D244" t="n">
+      <c r="D244" s="1" t="n">
         <v>40.200405</v>
       </c>
-      <c r="E244" t="n">
+      <c r="E244" s="1" t="n">
         <v>29.0544</v>
       </c>
-      <c r="F244" t="inlineStr">
+      <c r="F244" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -7221,28 +7239,28 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" t="inlineStr">
+      <c r="A247" s="1" t="inlineStr">
         <is>
           <t>R247HM</t>
         </is>
       </c>
-      <c r="B247" t="inlineStr">
+      <c r="B247" s="1" t="inlineStr">
         <is>
           <t>Umurbey Mahallesi, Cıngıllı Sokak, No: 6, Bursa</t>
         </is>
       </c>
-      <c r="C247" t="inlineStr">
+      <c r="C247" s="1" t="inlineStr">
         <is>
           <t>Davutkadı Mah., Çıngıllı Sok., No:6, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D247" t="n">
+      <c r="D247" s="1" t="n">
         <v>40.183313</v>
       </c>
-      <c r="E247" t="n">
+      <c r="E247" s="1" t="n">
         <v>29.085293</v>
       </c>
-      <c r="F247" t="inlineStr">
+      <c r="F247" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -7697,28 +7715,28 @@
       </c>
     </row>
     <row r="264">
-      <c r="A264" t="inlineStr">
+      <c r="A264" s="1" t="inlineStr">
         <is>
           <t>B264OB</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
+      <c r="B264" s="1" t="inlineStr">
         <is>
           <t>Millet Mahallesi, Kısmet Caddesi, No: 68, Bursa</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr">
+      <c r="C264" s="1" t="inlineStr">
         <is>
           <t>Kısmet Cad., No:68, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D264" t="n">
+      <c r="D264" s="1" t="n">
         <v>40.206149</v>
       </c>
-      <c r="E264" t="n">
+      <c r="E264" s="1" t="n">
         <v>29.0915</v>
       </c>
-      <c r="F264" t="inlineStr">
+      <c r="F264" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -7753,56 +7771,56 @@
       </c>
     </row>
     <row r="266">
-      <c r="A266" t="inlineStr">
+      <c r="A266" s="3" t="inlineStr">
         <is>
           <t>Z266RM</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
+      <c r="B266" s="3" t="inlineStr">
         <is>
           <t>Kapaklı Mahallesi, Kapaklı Sokak, No: 70, Bursa</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="C266" s="3" t="inlineStr">
         <is>
           <t>Kapaklı Mah., Kapaklı Sok., No:70, Akhisar, Manisa, Türkiye</t>
         </is>
       </c>
-      <c r="D266" t="n">
+      <c r="D266" s="3" t="n">
         <v>38.866843</v>
       </c>
-      <c r="E266" t="n">
+      <c r="E266" s="3" t="n">
         <v>27.744252</v>
       </c>
-      <c r="F266" t="inlineStr">
+      <c r="F266" s="3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="267">
-      <c r="A267" t="inlineStr">
+      <c r="A267" s="1" t="inlineStr">
         <is>
           <t>V267ZM</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
+      <c r="B267" s="1" t="inlineStr">
         <is>
           <t>Fidyekızık Mahallesi, Bursa Caddesi, No: 33, Bursa</t>
         </is>
       </c>
-      <c r="C267" t="inlineStr">
+      <c r="C267" s="1" t="inlineStr">
         <is>
           <t>Bursa Cad., No:33, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D267" t="n">
+      <c r="D267" s="1" t="n">
         <v>40.177918</v>
       </c>
-      <c r="E267" t="n">
+      <c r="E267" s="1" t="n">
         <v>29.134449</v>
       </c>
-      <c r="F267" t="inlineStr">
+      <c r="F267" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -7837,20 +7855,20 @@
       </c>
     </row>
     <row r="269">
-      <c r="A269" t="inlineStr">
+      <c r="A269" s="2" t="inlineStr">
         <is>
           <t>I269MM</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
+      <c r="B269" s="2" t="inlineStr">
         <is>
           <t>Gündoğdu Mahallesi, Örnek Site Caddesi, No: 6, Bursa</t>
         </is>
       </c>
-      <c r="C269" t="inlineStr"/>
-      <c r="D269" t="inlineStr"/>
-      <c r="E269" t="inlineStr"/>
-      <c r="F269" t="inlineStr">
+      <c r="C269" s="2" t="inlineStr"/>
+      <c r="D269" s="2" t="inlineStr"/>
+      <c r="E269" s="2" t="inlineStr"/>
+      <c r="F269" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -8305,56 +8323,56 @@
       </c>
     </row>
     <row r="286">
-      <c r="A286" t="inlineStr">
+      <c r="A286" s="3" t="inlineStr">
         <is>
           <t>I286OB</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B286" s="3" t="inlineStr">
         <is>
           <t>Yunusemre Mahallesi, Edip Sokak, No: 2A, Bursa</t>
         </is>
       </c>
-      <c r="C286" t="inlineStr">
+      <c r="C286" s="3" t="inlineStr">
         <is>
           <t>Yunusemre Mah., Edip Sok., No:2A, Zile, Tokat, Türkiye</t>
         </is>
       </c>
-      <c r="D286" t="n">
+      <c r="D286" s="3" t="n">
         <v>40.297197</v>
       </c>
-      <c r="E286" t="n">
+      <c r="E286" s="3" t="n">
         <v>35.870367</v>
       </c>
-      <c r="F286" t="inlineStr">
+      <c r="F286" s="3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
     </row>
     <row r="287">
-      <c r="A287" t="inlineStr">
+      <c r="A287" s="1" t="inlineStr">
         <is>
           <t>X287RM</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr">
+      <c r="B287" s="1" t="inlineStr">
         <is>
           <t>Sıracevizler Mahallesi, 4. Taşlı Sokak, No: 65, Bursa</t>
         </is>
       </c>
-      <c r="C287" t="inlineStr">
+      <c r="C287" s="1" t="inlineStr">
         <is>
           <t>4. Taşlı Sok., No:65, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D287" t="n">
+      <c r="D287" s="1" t="n">
         <v>40.179606</v>
       </c>
-      <c r="E287" t="n">
+      <c r="E287" s="1" t="n">
         <v>29.092722</v>
       </c>
-      <c r="F287" t="inlineStr">
+      <c r="F287" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -8837,20 +8855,20 @@
       </c>
     </row>
     <row r="305">
-      <c r="A305" t="inlineStr">
+      <c r="A305" s="2" t="inlineStr">
         <is>
           <t>Z305VM</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr">
+      <c r="B305" s="2" t="inlineStr">
         <is>
           <t>Balkan Mahallesi, Akçe Ağaç Caddesi, No: 2B, Bursa</t>
         </is>
       </c>
-      <c r="C305" t="inlineStr"/>
-      <c r="D305" t="inlineStr"/>
-      <c r="E305" t="inlineStr"/>
-      <c r="F305" t="inlineStr">
+      <c r="C305" s="2" t="inlineStr"/>
+      <c r="D305" s="2" t="inlineStr"/>
+      <c r="E305" s="2" t="inlineStr"/>
+      <c r="F305" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -9361,28 +9379,28 @@
       </c>
     </row>
     <row r="324">
-      <c r="A324" t="inlineStr">
+      <c r="A324" s="1" t="inlineStr">
         <is>
           <t>D324AB</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
+      <c r="B324" s="1" t="inlineStr">
         <is>
           <t>Kurtuluş Mahallesi, Şehit Cüneyt Yıldız Caddesi Çağlayan Sokak, No: 88, Bursa</t>
         </is>
       </c>
-      <c r="C324" t="inlineStr">
+      <c r="C324" s="1" t="inlineStr">
         <is>
           <t>Şehit Cüneyt Yıldız Cad., No:88, Gürsu, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D324" t="n">
+      <c r="D324" s="1" t="n">
         <v>40.214386</v>
       </c>
-      <c r="E324" t="n">
+      <c r="E324" s="1" t="n">
         <v>29.187252</v>
       </c>
-      <c r="F324" t="inlineStr">
+      <c r="F324" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -9613,20 +9631,20 @@
       </c>
     </row>
     <row r="333">
-      <c r="A333" t="inlineStr">
+      <c r="A333" s="2" t="inlineStr">
         <is>
           <t>G333IM</t>
         </is>
       </c>
-      <c r="B333" t="inlineStr">
+      <c r="B333" s="2" t="inlineStr">
         <is>
           <t>Vakıf Mahallesi, 2. Veda Sokak, No: 41, Bursa</t>
         </is>
       </c>
-      <c r="C333" t="inlineStr"/>
-      <c r="D333" t="inlineStr"/>
-      <c r="E333" t="inlineStr"/>
-      <c r="F333" t="inlineStr">
+      <c r="C333" s="2" t="inlineStr"/>
+      <c r="D333" s="2" t="inlineStr"/>
+      <c r="E333" s="2" t="inlineStr"/>
+      <c r="F333" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -9661,28 +9679,28 @@
       </c>
     </row>
     <row r="335">
-      <c r="A335" t="inlineStr">
+      <c r="A335" s="1" t="inlineStr">
         <is>
           <t>B335PM</t>
         </is>
       </c>
-      <c r="B335" t="inlineStr">
+      <c r="B335" s="1" t="inlineStr">
         <is>
           <t>Yunusemre Mahallesi, Kazımkarabekir Caddesi, No: 50, Bursa</t>
         </is>
       </c>
-      <c r="C335" t="inlineStr">
+      <c r="C335" s="1" t="inlineStr">
         <is>
           <t>Kazımkarabekir Cad., No:50, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D335" t="n">
+      <c r="D335" s="1" t="n">
         <v>40.200921</v>
       </c>
-      <c r="E335" t="n">
+      <c r="E335" s="1" t="n">
         <v>29.102145</v>
       </c>
-      <c r="F335" t="inlineStr">
+      <c r="F335" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -9717,28 +9735,28 @@
       </c>
     </row>
     <row r="337">
-      <c r="A337" t="inlineStr">
+      <c r="A337" s="1" t="inlineStr">
         <is>
           <t>M337YM</t>
         </is>
       </c>
-      <c r="B337" t="inlineStr">
+      <c r="B337" s="1" t="inlineStr">
         <is>
           <t>Erçeler Mahallesi, No: 290, Bursa</t>
         </is>
       </c>
-      <c r="C337" t="inlineStr">
+      <c r="C337" s="1" t="inlineStr">
         <is>
           <t>Epçeler Mah., Epçeler Bulunamayan Adresler Sok., No:290, Keles, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D337" t="n">
+      <c r="D337" s="1" t="n">
         <v>40.027371</v>
       </c>
-      <c r="E337" t="n">
+      <c r="E337" s="1" t="n">
         <v>29.234153</v>
       </c>
-      <c r="F337" t="inlineStr">
+      <c r="F337" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -9773,40 +9791,40 @@
       </c>
     </row>
     <row r="339">
-      <c r="A339" t="inlineStr">
+      <c r="A339" s="2" t="inlineStr">
         <is>
           <t>J339OB</t>
         </is>
       </c>
-      <c r="B339" t="inlineStr">
+      <c r="B339" s="2" t="inlineStr">
         <is>
           <t>Yunuseli Mahallesi, 842. Sokak, No: 3, Osmangazi, Bursa</t>
         </is>
       </c>
-      <c r="C339" t="inlineStr"/>
-      <c r="D339" t="inlineStr"/>
-      <c r="E339" t="inlineStr"/>
-      <c r="F339" t="inlineStr">
+      <c r="C339" s="2" t="inlineStr"/>
+      <c r="D339" s="2" t="inlineStr"/>
+      <c r="E339" s="2" t="inlineStr"/>
+      <c r="F339" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
     </row>
     <row r="340">
-      <c r="A340" t="inlineStr">
+      <c r="A340" s="2" t="inlineStr">
         <is>
           <t>A340GM</t>
         </is>
       </c>
-      <c r="B340" t="inlineStr">
+      <c r="B340" s="2" t="inlineStr">
         <is>
           <t>Karapınar Mahallesi, C120. Sokak, No: 4, Bursa</t>
         </is>
       </c>
-      <c r="C340" t="inlineStr"/>
-      <c r="D340" t="inlineStr"/>
-      <c r="E340" t="inlineStr"/>
-      <c r="F340" t="inlineStr">
+      <c r="C340" s="2" t="inlineStr"/>
+      <c r="D340" s="2" t="inlineStr"/>
+      <c r="E340" s="2" t="inlineStr"/>
+      <c r="F340" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -9953,20 +9971,20 @@
       </c>
     </row>
     <row r="346">
-      <c r="A346" t="inlineStr">
+      <c r="A346" s="2" t="inlineStr">
         <is>
           <t>O346KM</t>
         </is>
       </c>
-      <c r="B346" t="inlineStr">
+      <c r="B346" s="2" t="inlineStr">
         <is>
           <t>Alaaddin Mahallesi, Ortapazar Mahmutoğlu Sokak, No: 70, Bursa</t>
         </is>
       </c>
-      <c r="C346" t="inlineStr"/>
-      <c r="D346" t="inlineStr"/>
-      <c r="E346" t="inlineStr"/>
-      <c r="F346" t="inlineStr">
+      <c r="C346" s="2" t="inlineStr"/>
+      <c r="D346" s="2" t="inlineStr"/>
+      <c r="E346" s="2" t="inlineStr"/>
+      <c r="F346" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -10309,48 +10327,48 @@
       </c>
     </row>
     <row r="359">
-      <c r="A359" t="inlineStr">
+      <c r="A359" s="2" t="inlineStr">
         <is>
           <t>K359QB</t>
         </is>
       </c>
-      <c r="B359" t="inlineStr">
+      <c r="B359" s="2" t="inlineStr">
         <is>
           <t>Subaşı Mahallesi, Seyfi Demirsoy Sokak, No: 2, Bursa</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr"/>
-      <c r="D359" t="inlineStr"/>
-      <c r="E359" t="inlineStr"/>
-      <c r="F359" t="inlineStr">
+      <c r="C359" s="2" t="inlineStr"/>
+      <c r="D359" s="2" t="inlineStr"/>
+      <c r="E359" s="2" t="inlineStr"/>
+      <c r="F359" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
       </c>
     </row>
     <row r="360">
-      <c r="A360" t="inlineStr">
+      <c r="A360" s="1" t="inlineStr">
         <is>
           <t>Z360TM</t>
         </is>
       </c>
-      <c r="B360" t="inlineStr">
+      <c r="B360" s="1" t="inlineStr">
         <is>
           <t>Kiremitçi Mahallesi, Celal Bayar Caddesi, No: 89, Bursa</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr">
+      <c r="C360" s="1" t="inlineStr">
         <is>
           <t>Celal Bayar Cad., No:89, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D360" t="n">
+      <c r="D360" s="1" t="n">
         <v>40.191443</v>
       </c>
-      <c r="E360" t="n">
+      <c r="E360" s="1" t="n">
         <v>29.066087</v>
       </c>
-      <c r="F360" t="inlineStr">
+      <c r="F360" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -10665,28 +10683,28 @@
       </c>
     </row>
     <row r="372">
-      <c r="A372" t="inlineStr">
+      <c r="A372" s="1" t="inlineStr">
         <is>
           <t>C372OM</t>
         </is>
       </c>
-      <c r="B372" t="inlineStr">
+      <c r="B372" s="1" t="inlineStr">
         <is>
           <t>Bağlarbaşı Mahallesi, Hürriyet Caddesi, No: 166, Bursa</t>
         </is>
       </c>
-      <c r="C372" t="inlineStr">
+      <c r="C372" s="1" t="inlineStr">
         <is>
           <t>1. Hürriyet Cad., No:164-166, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D372" t="n">
+      <c r="D372" s="1" t="n">
         <v>40.231739</v>
       </c>
-      <c r="E372" t="n">
+      <c r="E372" s="1" t="n">
         <v>28.98602</v>
       </c>
-      <c r="F372" t="inlineStr">
+      <c r="F372" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -10721,20 +10739,20 @@
       </c>
     </row>
     <row r="374">
-      <c r="A374" t="inlineStr">
+      <c r="A374" s="2" t="inlineStr">
         <is>
           <t>E374EM</t>
         </is>
       </c>
-      <c r="B374" t="inlineStr">
+      <c r="B374" s="2" t="inlineStr">
         <is>
           <t>Demetevler Mahallesi, Kurban Pazarı Caddesi, No: 18, Bursa</t>
         </is>
       </c>
-      <c r="C374" t="inlineStr"/>
-      <c r="D374" t="inlineStr"/>
-      <c r="E374" t="inlineStr"/>
-      <c r="F374" t="inlineStr">
+      <c r="C374" s="2" t="inlineStr"/>
+      <c r="D374" s="2" t="inlineStr"/>
+      <c r="E374" s="2" t="inlineStr"/>
+      <c r="F374" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -11469,28 +11487,28 @@
       </c>
     </row>
     <row r="401">
-      <c r="A401" t="inlineStr">
+      <c r="A401" s="1" t="inlineStr">
         <is>
           <t>Q401ZM</t>
         </is>
       </c>
-      <c r="B401" t="inlineStr">
+      <c r="B401" s="1" t="inlineStr">
         <is>
           <t>Erikli Mahallesi, Erikli Caddesi, No: 72, Bursa</t>
         </is>
       </c>
-      <c r="C401" t="inlineStr">
+      <c r="C401" s="1" t="inlineStr">
         <is>
           <t>Erikli Cad., No:72, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D401" t="n">
+      <c r="D401" s="1" t="n">
         <v>40.186172</v>
       </c>
-      <c r="E401" t="n">
+      <c r="E401" s="1" t="n">
         <v>29.141518</v>
       </c>
-      <c r="F401" t="inlineStr">
+      <c r="F401" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -11833,28 +11851,28 @@
       </c>
     </row>
     <row r="414">
-      <c r="A414" t="inlineStr">
+      <c r="A414" s="1" t="inlineStr">
         <is>
           <t>D414MB</t>
         </is>
       </c>
-      <c r="B414" t="inlineStr">
+      <c r="B414" s="1" t="inlineStr">
         <is>
           <t>Çırpan Mahallesi, Stadyum Caddesi, No: 38, Bursa</t>
         </is>
       </c>
-      <c r="C414" t="inlineStr">
+      <c r="C414" s="1" t="inlineStr">
         <is>
           <t>Gaziakdemir Mah., Stadyum Cad., No:38, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D414" t="n">
+      <c r="D414" s="1" t="n">
         <v>40.196327</v>
       </c>
-      <c r="E414" t="n">
+      <c r="E414" s="1" t="n">
         <v>29.049486</v>
       </c>
-      <c r="F414" t="inlineStr">
+      <c r="F414" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -11945,28 +11963,28 @@
       </c>
     </row>
     <row r="418">
-      <c r="A418" t="inlineStr">
+      <c r="A418" s="3" t="inlineStr">
         <is>
           <t>T418KB</t>
         </is>
       </c>
-      <c r="B418" t="inlineStr">
+      <c r="B418" s="3" t="inlineStr">
         <is>
           <t>Asmalıevler Mahallesi, 6624. Sokak, No: 10F, Bursa</t>
         </is>
       </c>
-      <c r="C418" t="inlineStr">
+      <c r="C418" s="3" t="inlineStr">
         <is>
           <t>Asmalıevler Mah., 6624. Sok., No:10F, Pamukkale, Denizli, Türkiye</t>
         </is>
       </c>
-      <c r="D418" t="n">
+      <c r="D418" s="3" t="n">
         <v>37.747183</v>
       </c>
-      <c r="E418" t="n">
+      <c r="E418" s="3" t="n">
         <v>29.109961</v>
       </c>
-      <c r="F418" t="inlineStr">
+      <c r="F418" s="3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -12589,28 +12607,28 @@
       </c>
     </row>
     <row r="441">
-      <c r="A441" t="inlineStr">
+      <c r="A441" s="1" t="inlineStr">
         <is>
           <t>Q441WB</t>
         </is>
       </c>
-      <c r="B441" t="inlineStr">
+      <c r="B441" s="1" t="inlineStr">
         <is>
           <t>Altınşehir Mahallesi, Muammer Aksoy Caddesi, Bursa</t>
         </is>
       </c>
-      <c r="C441" t="inlineStr">
+      <c r="C441" s="1" t="inlineStr">
         <is>
           <t>Muammer Aksoy Cad., Nilüfer, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D441" t="n">
+      <c r="D441" s="1" t="n">
         <v>40.225246</v>
       </c>
-      <c r="E441" t="n">
+      <c r="E441" s="1" t="n">
         <v>28.916491</v>
       </c>
-      <c r="F441" t="inlineStr">
+      <c r="F441" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -12925,20 +12943,20 @@
       </c>
     </row>
     <row r="453">
-      <c r="A453" t="inlineStr">
+      <c r="A453" s="2" t="inlineStr">
         <is>
           <t>S453MB</t>
         </is>
       </c>
-      <c r="B453" t="inlineStr">
+      <c r="B453" s="2" t="inlineStr">
         <is>
           <t>Demirtaş Cumhuriyet Mahallesi, Selviyolu 2. Sokak, No: 3, Bursa</t>
         </is>
       </c>
-      <c r="C453" t="inlineStr"/>
-      <c r="D453" t="inlineStr"/>
-      <c r="E453" t="inlineStr"/>
-      <c r="F453" t="inlineStr">
+      <c r="C453" s="2" t="inlineStr"/>
+      <c r="D453" s="2" t="inlineStr"/>
+      <c r="E453" s="2" t="inlineStr"/>
+      <c r="F453" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -13085,28 +13103,28 @@
       </c>
     </row>
     <row r="459">
-      <c r="A459" t="inlineStr">
+      <c r="A459" s="3" t="inlineStr">
         <is>
           <t>N459JM</t>
         </is>
       </c>
-      <c r="B459" t="inlineStr">
+      <c r="B459" s="3" t="inlineStr">
         <is>
           <t>Seydiköy Köyü, Merkez Mevkii Merkez Küme Evleri, No: 21, Bursa</t>
         </is>
       </c>
-      <c r="C459" t="inlineStr">
+      <c r="C459" s="3" t="inlineStr">
         <is>
           <t>Seydiköy Köyü, Seydiköy Küme Evler, No:21, Kütahya Merkez , Kütahya, Türkiye</t>
         </is>
       </c>
-      <c r="D459" t="n">
+      <c r="D459" s="3" t="n">
         <v>39.540333</v>
       </c>
-      <c r="E459" t="n">
+      <c r="E459" s="3" t="n">
         <v>30.126764</v>
       </c>
-      <c r="F459" t="inlineStr">
+      <c r="F459" s="3" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -13281,20 +13299,20 @@
       </c>
     </row>
     <row r="466">
-      <c r="A466" t="inlineStr">
+      <c r="A466" s="2" t="inlineStr">
         <is>
           <t>J466NB</t>
         </is>
       </c>
-      <c r="B466" t="inlineStr">
+      <c r="B466" s="2" t="inlineStr">
         <is>
           <t>Ertuğrul Mahallesi, Elmas Sokak, No: 17C, Bursa</t>
         </is>
       </c>
-      <c r="C466" t="inlineStr"/>
-      <c r="D466" t="inlineStr"/>
-      <c r="E466" t="inlineStr"/>
-      <c r="F466" t="inlineStr">
+      <c r="C466" s="2" t="inlineStr"/>
+      <c r="D466" s="2" t="inlineStr"/>
+      <c r="E466" s="2" t="inlineStr"/>
+      <c r="F466" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -13609,20 +13627,20 @@
       </c>
     </row>
     <row r="478">
-      <c r="A478" t="inlineStr">
+      <c r="A478" s="2" t="inlineStr">
         <is>
           <t>G478SM</t>
         </is>
       </c>
-      <c r="B478" t="inlineStr">
+      <c r="B478" s="2" t="inlineStr">
         <is>
           <t>Demetevler Mahallesi, İsmetiye Caddesi, No: 137, Bursa</t>
         </is>
       </c>
-      <c r="C478" t="inlineStr"/>
-      <c r="D478" t="inlineStr"/>
-      <c r="E478" t="inlineStr"/>
-      <c r="F478" t="inlineStr">
+      <c r="C478" s="2" t="inlineStr"/>
+      <c r="D478" s="2" t="inlineStr"/>
+      <c r="E478" s="2" t="inlineStr"/>
+      <c r="F478" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -13769,20 +13787,20 @@
       </c>
     </row>
     <row r="484">
-      <c r="A484" t="inlineStr">
+      <c r="A484" s="2" t="inlineStr">
         <is>
           <t>F484GM</t>
         </is>
       </c>
-      <c r="B484" t="inlineStr">
+      <c r="B484" s="2" t="inlineStr">
         <is>
           <t>Davutdede Mahallesi, 2. Güzel Sokak, No: 2, Bursa</t>
         </is>
       </c>
-      <c r="C484" t="inlineStr"/>
-      <c r="D484" t="inlineStr"/>
-      <c r="E484" t="inlineStr"/>
-      <c r="F484" t="inlineStr">
+      <c r="C484" s="2" t="inlineStr"/>
+      <c r="D484" s="2" t="inlineStr"/>
+      <c r="E484" s="2" t="inlineStr"/>
+      <c r="F484" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -14433,20 +14451,20 @@
       </c>
     </row>
     <row r="508">
-      <c r="A508" t="inlineStr">
+      <c r="A508" s="2" t="inlineStr">
         <is>
           <t>K508MB</t>
         </is>
       </c>
-      <c r="B508" t="inlineStr">
+      <c r="B508" s="2" t="inlineStr">
         <is>
           <t>Kırcaali Mahallesi, Aydoğmuş Sokak, No: 11, Bursa</t>
         </is>
       </c>
-      <c r="C508" t="inlineStr"/>
-      <c r="D508" t="inlineStr"/>
-      <c r="E508" t="inlineStr"/>
-      <c r="F508" t="inlineStr">
+      <c r="C508" s="2" t="inlineStr"/>
+      <c r="D508" s="2" t="inlineStr"/>
+      <c r="E508" s="2" t="inlineStr"/>
+      <c r="F508" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -14537,20 +14555,20 @@
       </c>
     </row>
     <row r="512">
-      <c r="A512" t="inlineStr">
+      <c r="A512" s="2" t="inlineStr">
         <is>
           <t>X512HB</t>
         </is>
       </c>
-      <c r="B512" t="inlineStr">
+      <c r="B512" s="2" t="inlineStr">
         <is>
           <t>Yunuseli Mahallesi, 842. Sokak, No: 3, Bursa</t>
         </is>
       </c>
-      <c r="C512" t="inlineStr"/>
-      <c r="D512" t="inlineStr"/>
-      <c r="E512" t="inlineStr"/>
-      <c r="F512" t="inlineStr">
+      <c r="C512" s="2" t="inlineStr"/>
+      <c r="D512" s="2" t="inlineStr"/>
+      <c r="E512" s="2" t="inlineStr"/>
+      <c r="F512" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -15089,28 +15107,28 @@
       </c>
     </row>
     <row r="532">
-      <c r="A532" t="inlineStr">
+      <c r="A532" s="1" t="inlineStr">
         <is>
           <t>T532HM</t>
         </is>
       </c>
-      <c r="B532" t="inlineStr">
+      <c r="B532" s="1" t="inlineStr">
         <is>
           <t>Güllük Mahallesi, Girne Caddesi, No: 110, Bursa</t>
         </is>
       </c>
-      <c r="C532" t="inlineStr">
+      <c r="C532" s="1" t="inlineStr">
         <is>
           <t>Girne Cad., No:110, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D532" t="n">
+      <c r="D532" s="1" t="n">
         <v>40.185752</v>
       </c>
-      <c r="E532" t="n">
+      <c r="E532" s="1" t="n">
         <v>29.121486</v>
       </c>
-      <c r="F532" t="inlineStr">
+      <c r="F532" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -15761,28 +15779,28 @@
       </c>
     </row>
     <row r="556">
-      <c r="A556" t="inlineStr">
+      <c r="A556" s="1" t="inlineStr">
         <is>
           <t>U556YM</t>
         </is>
       </c>
-      <c r="B556" t="inlineStr">
+      <c r="B556" s="1" t="inlineStr">
         <is>
           <t>Çiftehavuzlar Mahallesi, Özcan Caddesi, No: 56, Bursa</t>
         </is>
       </c>
-      <c r="C556" t="inlineStr">
+      <c r="C556" s="1" t="inlineStr">
         <is>
           <t>Özcan Cad., No:56, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D556" t="n">
+      <c r="D556" s="1" t="n">
         <v>40.211501</v>
       </c>
-      <c r="E556" t="n">
+      <c r="E556" s="1" t="n">
         <v>29.054292</v>
       </c>
-      <c r="F556" t="inlineStr">
+      <c r="F556" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -16097,20 +16115,20 @@
       </c>
     </row>
     <row r="568">
-      <c r="A568" t="inlineStr">
+      <c r="A568" s="2" t="inlineStr">
         <is>
           <t>H568VM</t>
         </is>
       </c>
-      <c r="B568" t="inlineStr">
+      <c r="B568" s="2" t="inlineStr">
         <is>
           <t>Ovaakça Merkez Mahallesi, Kürşat Sokak, No: 1, Bursa</t>
         </is>
       </c>
-      <c r="C568" t="inlineStr"/>
-      <c r="D568" t="inlineStr"/>
-      <c r="E568" t="inlineStr"/>
-      <c r="F568" t="inlineStr">
+      <c r="C568" s="2" t="inlineStr"/>
+      <c r="D568" s="2" t="inlineStr"/>
+      <c r="E568" s="2" t="inlineStr"/>
+      <c r="F568" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -16341,20 +16359,20 @@
       </c>
     </row>
     <row r="577">
-      <c r="A577" t="inlineStr">
+      <c r="A577" s="2" t="inlineStr">
         <is>
           <t>S577ZM</t>
         </is>
       </c>
-      <c r="B577" t="inlineStr">
+      <c r="B577" s="2" t="inlineStr">
         <is>
           <t>Değirmenönü Mahallesi, Şehitler Caddesi, No: 17A, Bursa</t>
         </is>
       </c>
-      <c r="C577" t="inlineStr"/>
-      <c r="D577" t="inlineStr"/>
-      <c r="E577" t="inlineStr"/>
-      <c r="F577" t="inlineStr">
+      <c r="C577" s="2" t="inlineStr"/>
+      <c r="D577" s="2" t="inlineStr"/>
+      <c r="E577" s="2" t="inlineStr"/>
+      <c r="F577" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -16669,28 +16687,28 @@
       </c>
     </row>
     <row r="589">
-      <c r="A589" t="inlineStr">
+      <c r="A589" s="1" t="inlineStr">
         <is>
           <t>S589TM</t>
         </is>
       </c>
-      <c r="B589" t="inlineStr">
+      <c r="B589" s="1" t="inlineStr">
         <is>
           <t>Yavuzselim Mahallesi, Barış Caddesi, No: 42, Bursa</t>
         </is>
       </c>
-      <c r="C589" t="inlineStr">
+      <c r="C589" s="1" t="inlineStr">
         <is>
           <t>Barış Cad., No:42, Yıldırım, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D589" t="n">
+      <c r="D589" s="1" t="n">
         <v>40.194481</v>
       </c>
-      <c r="E589" t="n">
+      <c r="E589" s="1" t="n">
         <v>29.111128</v>
       </c>
-      <c r="F589" t="inlineStr">
+      <c r="F589" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
@@ -16809,20 +16827,20 @@
       </c>
     </row>
     <row r="594">
-      <c r="A594" t="inlineStr">
+      <c r="A594" s="2" t="inlineStr">
         <is>
           <t>U594UB</t>
         </is>
       </c>
-      <c r="B594" t="inlineStr">
+      <c r="B594" s="2" t="inlineStr">
         <is>
           <t>Balkan Mahallesi, Köseler Caddesi, No: 4C, Bursa</t>
         </is>
       </c>
-      <c r="C594" t="inlineStr"/>
-      <c r="D594" t="inlineStr"/>
-      <c r="E594" t="inlineStr"/>
-      <c r="F594" t="inlineStr">
+      <c r="C594" s="2" t="inlineStr"/>
+      <c r="D594" s="2" t="inlineStr"/>
+      <c r="E594" s="2" t="inlineStr"/>
+      <c r="F594" s="2" t="inlineStr">
         <is>
           <t>failed</t>
         </is>
@@ -16857,28 +16875,28 @@
       </c>
     </row>
     <row r="596">
-      <c r="A596" t="inlineStr">
+      <c r="A596" s="1" t="inlineStr">
         <is>
           <t>O596QM</t>
         </is>
       </c>
-      <c r="B596" t="inlineStr">
+      <c r="B596" s="1" t="inlineStr">
         <is>
           <t>Demirtaş Cumhuriyet Mahallesi, Küçük Sanayi Caddesi, No: 51, Bursa</t>
         </is>
       </c>
-      <c r="C596" t="inlineStr">
+      <c r="C596" s="1" t="inlineStr">
         <is>
           <t>Cumhuriyet Cad., No:51, Osmangazi, Bursa, Türkiye</t>
         </is>
       </c>
-      <c r="D596" t="n">
+      <c r="D596" s="1" t="n">
         <v>40.185277</v>
       </c>
-      <c r="E596" t="n">
+      <c r="E596" s="1" t="n">
         <v>29.068243</v>
       </c>
-      <c r="F596" t="inlineStr">
+      <c r="F596" s="1" t="inlineStr">
         <is>
           <t>ok</t>
         </is>

</xml_diff>